<commit_message>
Continue development: operator identification ; cancellations status correction
</commit_message>
<xml_diff>
--- a/summary_stats/chuuchuu_summary_full_2025_april.xlsx
+++ b/summary_stats/chuuchuu_summary_full_2025_april.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M128"/>
+  <dimension ref="A1:M129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -525,13 +525,13 @@
         <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="M2" t="n">
-        <v>0</v>
+        <v>142</v>
       </c>
     </row>
     <row r="3">
@@ -582,7 +582,7 @@
         <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>0</v>
+        <v>149</v>
       </c>
     </row>
     <row r="4">
@@ -672,19 +672,19 @@
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
+        <v>107</v>
       </c>
     </row>
     <row r="6">
@@ -729,13 +729,13 @@
         <v>1</v>
       </c>
       <c r="K6" t="n">
-        <v>1</v>
+        <v>65</v>
       </c>
       <c r="L6" t="n">
-        <v>1</v>
+        <v>28</v>
       </c>
       <c r="M6" t="n">
-        <v>1</v>
+        <v>397</v>
       </c>
     </row>
     <row r="7">
@@ -780,13 +780,13 @@
         <v>1</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -825,19 +825,19 @@
         <v>1</v>
       </c>
       <c r="I8" t="n">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="J8" t="n">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="K8" t="n">
-        <v>6</v>
+        <v>268</v>
       </c>
       <c r="L8" t="n">
-        <v>5</v>
+        <v>119</v>
       </c>
       <c r="M8" t="n">
-        <v>7</v>
+        <v>621</v>
       </c>
     </row>
     <row r="9">
@@ -876,19 +876,19 @@
         <v>1</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="L9" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="M9" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10">
@@ -927,19 +927,19 @@
         <v>110</v>
       </c>
       <c r="I10" t="n">
-        <v>157</v>
+        <v>402</v>
       </c>
       <c r="J10" t="n">
-        <v>267</v>
+        <v>512</v>
       </c>
       <c r="K10" t="n">
-        <v>39</v>
+        <v>1913</v>
       </c>
       <c r="L10" t="n">
-        <v>29</v>
+        <v>982</v>
       </c>
       <c r="M10" t="n">
-        <v>47</v>
+        <v>4054</v>
       </c>
     </row>
     <row r="11">
@@ -978,19 +978,19 @@
         <v>2</v>
       </c>
       <c r="I11" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="J11" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="K11" t="n">
-        <v>3</v>
+        <v>130</v>
       </c>
       <c r="L11" t="n">
-        <v>3</v>
+        <v>87</v>
       </c>
       <c r="M11" t="n">
-        <v>10</v>
+        <v>249</v>
       </c>
     </row>
     <row r="12">
@@ -999,22 +999,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>DSB</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>IC</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>domestic</t>
+          <t>international</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1023,25 +1023,25 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>13744</v>
+        <v>405</v>
       </c>
       <c r="H12" t="n">
-        <v>568</v>
+        <v>2</v>
       </c>
       <c r="I12" t="n">
-        <v>449</v>
+        <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>1017</v>
+        <v>2</v>
       </c>
       <c r="K12" t="n">
-        <v>170</v>
+        <v>58</v>
       </c>
       <c r="L12" t="n">
-        <v>159</v>
+        <v>8</v>
       </c>
       <c r="M12" t="n">
-        <v>188</v>
+        <v>403</v>
       </c>
     </row>
     <row r="13">
@@ -1050,7 +1050,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>Deutsche Bahn</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1060,7 +1060,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>international</t>
+          <t>domestic</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1070,29 +1070,29 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>1538</v>
+        <v>13744</v>
       </c>
       <c r="H13" t="n">
-        <v>39</v>
+        <v>568</v>
       </c>
       <c r="I13" t="n">
-        <v>58</v>
+        <v>1099</v>
       </c>
       <c r="J13" t="n">
-        <v>97</v>
+        <v>1667</v>
       </c>
       <c r="K13" t="n">
-        <v>216</v>
+        <v>6941</v>
       </c>
       <c r="L13" t="n">
-        <v>106</v>
+        <v>4050</v>
       </c>
       <c r="M13" t="n">
-        <v>513</v>
+        <v>12876</v>
       </c>
     </row>
     <row r="14">
@@ -1101,7 +1101,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>DB</t>
+          <t>Deutsche Bahn</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1111,7 +1111,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>international</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -1121,29 +1121,29 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>47</v>
+        <v>1538</v>
       </c>
       <c r="H14" t="n">
-        <v>1</v>
+        <v>39</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
+        <v>81</v>
       </c>
       <c r="J14" t="n">
-        <v>1</v>
+        <v>120</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>448</v>
       </c>
       <c r="L14" t="n">
-        <v>0</v>
+        <v>241</v>
       </c>
       <c r="M14" t="n">
-        <v>0</v>
+        <v>1072</v>
       </c>
     </row>
     <row r="15">
@@ -1152,40 +1152,40 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>DSB</t>
+          <t>Deutsche Bahn</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>IC</t>
+          <t>ICE</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>international</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>405</v>
+        <v>47</v>
       </c>
       <c r="H15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I15" t="n">
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
@@ -1290,13 +1290,13 @@
         <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="L17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="M17" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
     </row>
     <row r="18">
@@ -1386,19 +1386,19 @@
         <v>6</v>
       </c>
       <c r="I19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J19" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K19" t="n">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="L19" t="n">
-        <v>12</v>
+        <v>23</v>
       </c>
       <c r="M19" t="n">
-        <v>17</v>
+        <v>29</v>
       </c>
     </row>
     <row r="20">
@@ -1437,19 +1437,19 @@
         <v>6</v>
       </c>
       <c r="I20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J20" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K20" t="n">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="L20" t="n">
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="M20" t="n">
-        <v>16</v>
+        <v>28</v>
       </c>
     </row>
     <row r="21">
@@ -1539,19 +1539,19 @@
         <v>1</v>
       </c>
       <c r="I22" t="n">
-        <v>4</v>
+        <v>32</v>
       </c>
       <c r="J22" t="n">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="K22" t="n">
-        <v>3</v>
+        <v>292</v>
       </c>
       <c r="L22" t="n">
-        <v>3</v>
+        <v>188</v>
       </c>
       <c r="M22" t="n">
-        <v>3</v>
+        <v>468</v>
       </c>
     </row>
     <row r="23">
@@ -1641,19 +1641,19 @@
         <v>0</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J24" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K24" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="L24" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M24" t="n">
-        <v>0</v>
+        <v>58</v>
       </c>
     </row>
     <row r="25">
@@ -1692,19 +1692,19 @@
         <v>7</v>
       </c>
       <c r="I25" t="n">
-        <v>12</v>
+        <v>4981</v>
       </c>
       <c r="J25" t="n">
-        <v>19</v>
+        <v>4988</v>
       </c>
       <c r="K25" t="n">
-        <v>0</v>
+        <v>1831</v>
       </c>
       <c r="L25" t="n">
-        <v>0</v>
+        <v>360</v>
       </c>
       <c r="M25" t="n">
-        <v>0</v>
+        <v>26511</v>
       </c>
     </row>
     <row r="26">
@@ -1845,19 +1845,19 @@
         <v>0</v>
       </c>
       <c r="I28" t="n">
-        <v>4</v>
+        <v>668</v>
       </c>
       <c r="J28" t="n">
-        <v>4</v>
+        <v>668</v>
       </c>
       <c r="K28" t="n">
-        <v>0</v>
+        <v>302</v>
       </c>
       <c r="L28" t="n">
-        <v>0</v>
+        <v>68</v>
       </c>
       <c r="M28" t="n">
-        <v>0</v>
+        <v>2272</v>
       </c>
     </row>
     <row r="29">
@@ -1947,19 +1947,19 @@
         <v>0</v>
       </c>
       <c r="I30" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J30" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="K30" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L30" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M30" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="31">
@@ -1998,19 +1998,19 @@
         <v>43</v>
       </c>
       <c r="I31" t="n">
-        <v>43</v>
+        <v>632</v>
       </c>
       <c r="J31" t="n">
-        <v>86</v>
+        <v>675</v>
       </c>
       <c r="K31" t="n">
-        <v>84</v>
+        <v>256</v>
       </c>
       <c r="L31" t="n">
-        <v>16</v>
+        <v>68</v>
       </c>
       <c r="M31" t="n">
-        <v>877</v>
+        <v>4522</v>
       </c>
     </row>
     <row r="32">
@@ -2049,10 +2049,10 @@
         <v>0</v>
       </c>
       <c r="I32" t="n">
-        <v>0</v>
+        <v>178</v>
       </c>
       <c r="J32" t="n">
-        <v>0</v>
+        <v>178</v>
       </c>
       <c r="K32" t="n">
         <v>0</v>
@@ -2151,19 +2151,19 @@
         <v>0</v>
       </c>
       <c r="I34" t="n">
-        <v>10</v>
+        <v>8093</v>
       </c>
       <c r="J34" t="n">
-        <v>10</v>
+        <v>8093</v>
       </c>
       <c r="K34" t="n">
-        <v>0</v>
+        <v>1986</v>
       </c>
       <c r="L34" t="n">
-        <v>0</v>
+        <v>283</v>
       </c>
       <c r="M34" t="n">
-        <v>0</v>
+        <v>61150</v>
       </c>
     </row>
     <row r="35">
@@ -2253,19 +2253,19 @@
         <v>121</v>
       </c>
       <c r="I36" t="n">
-        <v>2</v>
+        <v>3872</v>
       </c>
       <c r="J36" t="n">
-        <v>123</v>
+        <v>3993</v>
       </c>
       <c r="K36" t="n">
-        <v>33</v>
+        <v>865</v>
       </c>
       <c r="L36" t="n">
-        <v>13</v>
+        <v>177</v>
       </c>
       <c r="M36" t="n">
-        <v>843</v>
+        <v>32968</v>
       </c>
     </row>
     <row r="37">
@@ -2304,10 +2304,10 @@
         <v>0</v>
       </c>
       <c r="I37" t="n">
-        <v>0</v>
+        <v>213</v>
       </c>
       <c r="J37" t="n">
-        <v>0</v>
+        <v>213</v>
       </c>
       <c r="K37" t="n">
         <v>0</v>
@@ -2406,19 +2406,19 @@
         <v>4</v>
       </c>
       <c r="I39" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="J39" t="n">
+        <v>19</v>
+      </c>
+      <c r="K39" t="n">
+        <v>68</v>
+      </c>
+      <c r="L39" t="n">
         <v>17</v>
       </c>
-      <c r="K39" t="n">
-        <v>0</v>
-      </c>
-      <c r="L39" t="n">
-        <v>0</v>
-      </c>
       <c r="M39" t="n">
-        <v>0</v>
+        <v>706</v>
       </c>
     </row>
     <row r="40">
@@ -2463,13 +2463,13 @@
         <v>1</v>
       </c>
       <c r="K40" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="L40" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="M40" t="n">
-        <v>0</v>
+        <v>281</v>
       </c>
     </row>
     <row r="41">
@@ -2514,13 +2514,13 @@
         <v>0</v>
       </c>
       <c r="K41" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="L41" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="M41" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
     </row>
     <row r="42">
@@ -2559,19 +2559,19 @@
         <v>0</v>
       </c>
       <c r="I42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K42" t="n">
-        <v>0</v>
+        <v>187</v>
       </c>
       <c r="L42" t="n">
-        <v>0</v>
+        <v>128</v>
       </c>
       <c r="M42" t="n">
-        <v>0</v>
+        <v>632</v>
       </c>
     </row>
     <row r="43">
@@ -2616,13 +2616,13 @@
         <v>0</v>
       </c>
       <c r="K43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L43" t="n">
         <v>0</v>
       </c>
       <c r="M43" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="44">
@@ -2661,19 +2661,19 @@
         <v>3</v>
       </c>
       <c r="I44" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J44" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="K44" t="n">
-        <v>1</v>
+        <v>164</v>
       </c>
       <c r="L44" t="n">
-        <v>1</v>
+        <v>51</v>
       </c>
       <c r="M44" t="n">
-        <v>1</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="45">
@@ -2718,13 +2718,13 @@
         <v>0</v>
       </c>
       <c r="K45" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M45" t="n">
-        <v>0</v>
+        <v>113</v>
       </c>
     </row>
     <row r="46">
@@ -2763,19 +2763,19 @@
         <v>2</v>
       </c>
       <c r="I46" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J46" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K46" t="n">
-        <v>51</v>
+        <v>81</v>
       </c>
       <c r="L46" t="n">
-        <v>29</v>
+        <v>57</v>
       </c>
       <c r="M46" t="n">
-        <v>85</v>
+        <v>179</v>
       </c>
     </row>
     <row r="47">
@@ -2814,19 +2814,19 @@
         <v>1</v>
       </c>
       <c r="I47" t="n">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="J47" t="n">
-        <v>6</v>
+        <v>41</v>
       </c>
       <c r="K47" t="n">
-        <v>16</v>
+        <v>62</v>
       </c>
       <c r="L47" t="n">
-        <v>13</v>
+        <v>39</v>
       </c>
       <c r="M47" t="n">
-        <v>46</v>
+        <v>291</v>
       </c>
     </row>
     <row r="48">
@@ -2916,19 +2916,19 @@
         <v>4</v>
       </c>
       <c r="I49" t="n">
-        <v>31</v>
+        <v>61</v>
       </c>
       <c r="J49" t="n">
-        <v>35</v>
+        <v>65</v>
       </c>
       <c r="K49" t="n">
-        <v>7</v>
+        <v>189</v>
       </c>
       <c r="L49" t="n">
-        <v>7</v>
+        <v>52</v>
       </c>
       <c r="M49" t="n">
-        <v>7</v>
+        <v>1817</v>
       </c>
     </row>
     <row r="50">
@@ -2973,13 +2973,13 @@
         <v>0</v>
       </c>
       <c r="K50" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="L50" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="M50" t="n">
-        <v>0</v>
+        <v>115</v>
       </c>
     </row>
     <row r="51">
@@ -3018,19 +3018,19 @@
         <v>2</v>
       </c>
       <c r="I51" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="J51" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="K51" t="n">
-        <v>2</v>
+        <v>254</v>
       </c>
       <c r="L51" t="n">
-        <v>2</v>
+        <v>126</v>
       </c>
       <c r="M51" t="n">
-        <v>3</v>
+        <v>886</v>
       </c>
     </row>
     <row r="52">
@@ -3069,19 +3069,19 @@
         <v>0</v>
       </c>
       <c r="I52" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="J52" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="K52" t="n">
-        <v>0</v>
+        <v>76</v>
       </c>
       <c r="L52" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="M52" t="n">
-        <v>1</v>
+        <v>242</v>
       </c>
     </row>
     <row r="53">
@@ -3234,7 +3234,7 @@
         <v>0</v>
       </c>
       <c r="M55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="56">
@@ -3273,19 +3273,19 @@
         <v>1</v>
       </c>
       <c r="I56" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J56" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="K56" t="n">
-        <v>3</v>
+        <v>241</v>
       </c>
       <c r="L56" t="n">
-        <v>3</v>
+        <v>126</v>
       </c>
       <c r="M56" t="n">
-        <v>3</v>
+        <v>642</v>
       </c>
     </row>
     <row r="57">
@@ -3330,13 +3330,13 @@
         <v>1</v>
       </c>
       <c r="K57" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L57" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M57" t="n">
-        <v>156</v>
+        <v>206</v>
       </c>
     </row>
     <row r="58">
@@ -3375,19 +3375,19 @@
         <v>5</v>
       </c>
       <c r="I58" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J58" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K58" t="n">
-        <v>7</v>
+        <v>42</v>
       </c>
       <c r="L58" t="n">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="M58" t="n">
-        <v>105</v>
+        <v>688</v>
       </c>
     </row>
     <row r="59">
@@ -3426,19 +3426,19 @@
         <v>1</v>
       </c>
       <c r="I59" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J59" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K59" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="L59" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="M59" t="n">
-        <v>1</v>
+        <v>59</v>
       </c>
     </row>
     <row r="60">
@@ -3477,19 +3477,19 @@
         <v>15</v>
       </c>
       <c r="I60" t="n">
-        <v>127</v>
+        <v>139</v>
       </c>
       <c r="J60" t="n">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="K60" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="L60" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="M60" t="n">
-        <v>1</v>
+        <v>10575</v>
       </c>
     </row>
     <row r="61">
@@ -3534,13 +3534,13 @@
         <v>0</v>
       </c>
       <c r="K61" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L61" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M61" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
     </row>
     <row r="62">
@@ -3630,19 +3630,19 @@
         <v>28</v>
       </c>
       <c r="I63" t="n">
-        <v>112</v>
+        <v>148</v>
       </c>
       <c r="J63" t="n">
-        <v>140</v>
+        <v>176</v>
       </c>
       <c r="K63" t="n">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="L63" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="M63" t="n">
-        <v>4</v>
+        <v>11998</v>
       </c>
     </row>
     <row r="64">
@@ -3681,19 +3681,19 @@
         <v>0</v>
       </c>
       <c r="I64" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="J64" t="n">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="K64" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="L64" t="n">
         <v>0</v>
       </c>
       <c r="M64" t="n">
-        <v>0</v>
+        <v>821</v>
       </c>
     </row>
     <row r="65">
@@ -3789,13 +3789,13 @@
         <v>2</v>
       </c>
       <c r="K66" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="L66" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="M66" t="n">
-        <v>0</v>
+        <v>43</v>
       </c>
     </row>
     <row r="67">
@@ -4314,12 +4314,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>SNCF</t>
+          <t>SNCB/NS</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>INTERCITES</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -4334,29 +4334,29 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G77" t="n">
-        <v>2050</v>
+        <v>1</v>
       </c>
       <c r="H77" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="I77" t="n">
-        <v>19</v>
+        <v>0</v>
       </c>
       <c r="J77" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="K77" t="n">
-        <v>425</v>
+        <v>1</v>
       </c>
       <c r="L77" t="n">
-        <v>268</v>
+        <v>1</v>
       </c>
       <c r="M77" t="n">
-        <v>2033</v>
+        <v>1</v>
       </c>
     </row>
     <row r="78">
@@ -4365,17 +4365,17 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>SNCF</t>
+          <t>SNCB/NS</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>INTERCITES DE NUIT</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>domestic</t>
+          <t>international</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -4385,29 +4385,29 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G78" t="n">
-        <v>248</v>
+        <v>696</v>
       </c>
       <c r="H78" t="n">
         <v>0</v>
       </c>
       <c r="I78" t="n">
-        <v>3</v>
+        <v>32</v>
       </c>
       <c r="J78" t="n">
-        <v>3</v>
+        <v>32</v>
       </c>
       <c r="K78" t="n">
-        <v>22</v>
+        <v>128</v>
       </c>
       <c r="L78" t="n">
-        <v>12</v>
+        <v>46</v>
       </c>
       <c r="M78" t="n">
-        <v>247</v>
+        <v>686</v>
       </c>
     </row>
     <row r="79">
@@ -4416,22 +4416,22 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>SNCF</t>
+          <t>SNCB/NS</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>LYRIA</t>
+          <t>ECC</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>international</t>
+          <t>domestic</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -4440,25 +4440,25 @@
         </is>
       </c>
       <c r="G79" t="n">
-        <v>1040</v>
+        <v>401</v>
       </c>
       <c r="H79" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="I79" t="n">
-        <v>5</v>
+        <v>83</v>
       </c>
       <c r="J79" t="n">
-        <v>5</v>
+        <v>128</v>
       </c>
       <c r="K79" t="n">
-        <v>112</v>
+        <v>47</v>
       </c>
       <c r="L79" t="n">
-        <v>56</v>
+        <v>23</v>
       </c>
       <c r="M79" t="n">
-        <v>1038</v>
+        <v>282</v>
       </c>
     </row>
     <row r="80">
@@ -4467,40 +4467,40 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>SNCF</t>
+          <t>SNCB/NS</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>TGV</t>
+          <t>ECC</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>domestic</t>
+          <t>international</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G80" t="n">
-        <v>53</v>
+        <v>64</v>
       </c>
       <c r="H80" t="n">
         <v>0</v>
       </c>
       <c r="I80" t="n">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="J80" t="n">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="K80" t="n">
         <v>0</v>
@@ -4518,49 +4518,49 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>SNCF</t>
+          <t>SNCB/NS</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>TGV</t>
+          <t>ECC</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>international</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G81" t="n">
-        <v>1343</v>
+        <v>317</v>
       </c>
       <c r="H81" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="I81" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J81" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="K81" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L81" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M81" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="82">
@@ -4569,12 +4569,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>SNCF</t>
+          <t>SNCB/NS</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>TGV INOUI</t>
+          <t>ECD</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -4584,34 +4584,34 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G82" t="n">
-        <v>14774</v>
+        <v>85</v>
       </c>
       <c r="H82" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="I82" t="n">
-        <v>129</v>
+        <v>12</v>
       </c>
       <c r="J82" t="n">
-        <v>146</v>
+        <v>30</v>
       </c>
       <c r="K82" t="n">
-        <v>2042</v>
+        <v>19</v>
       </c>
       <c r="L82" t="n">
-        <v>943</v>
+        <v>14</v>
       </c>
       <c r="M82" t="n">
-        <v>14714</v>
+        <v>45</v>
       </c>
     </row>
     <row r="83">
@@ -4620,12 +4620,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>SNCF</t>
+          <t>SNCB/NS</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>TGV INOUI</t>
+          <t>ECD</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -4635,34 +4635,34 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G83" t="n">
-        <v>1140</v>
+        <v>731</v>
       </c>
       <c r="H83" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="I83" t="n">
+        <v>15</v>
+      </c>
+      <c r="J83" t="n">
         <v>18</v>
       </c>
-      <c r="J83" t="n">
-        <v>25</v>
-      </c>
       <c r="K83" t="n">
-        <v>271</v>
+        <v>78</v>
       </c>
       <c r="L83" t="n">
-        <v>143</v>
+        <v>33</v>
       </c>
       <c r="M83" t="n">
-        <v>1122</v>
+        <v>541</v>
       </c>
     </row>
     <row r="84">
@@ -4671,17 +4671,17 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Trenitalia</t>
+          <t>SNCB/NS</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>EC</t>
+          <t>ECD</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>domestic</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -4695,25 +4695,25 @@
         </is>
       </c>
       <c r="G84" t="n">
-        <v>846</v>
+        <v>64</v>
       </c>
       <c r="H84" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I84" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J84" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="K84" t="n">
-        <v>180</v>
+        <v>0</v>
       </c>
       <c r="L84" t="n">
-        <v>64</v>
+        <v>0</v>
       </c>
       <c r="M84" t="n">
-        <v>837</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85">
@@ -4722,17 +4722,17 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Trenitalia</t>
+          <t>SNCF</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>EC</t>
+          <t>INTERCITES</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>domestic</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
@@ -4742,29 +4742,29 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G85" t="n">
-        <v>421</v>
+        <v>2050</v>
       </c>
       <c r="H85" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="I85" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="J85" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="K85" t="n">
-        <v>0</v>
+        <v>425</v>
       </c>
       <c r="L85" t="n">
-        <v>0</v>
+        <v>268</v>
       </c>
       <c r="M85" t="n">
-        <v>0</v>
+        <v>2033</v>
       </c>
     </row>
     <row r="86">
@@ -4773,12 +4773,12 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Trenitalia</t>
+          <t>SNCF</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>EN</t>
+          <t>INTERCITES DE NUIT</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -4793,29 +4793,29 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G86" t="n">
+        <v>248</v>
+      </c>
+      <c r="H86" t="n">
+        <v>0</v>
+      </c>
+      <c r="I86" t="n">
         <v>3</v>
       </c>
-      <c r="H86" t="n">
-        <v>0</v>
-      </c>
-      <c r="I86" t="n">
-        <v>0</v>
-      </c>
       <c r="J86" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K86" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="L86" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="M86" t="n">
-        <v>3</v>
+        <v>247</v>
       </c>
     </row>
     <row r="87">
@@ -4824,22 +4824,22 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Trenitalia</t>
+          <t>SNCF</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>EN</t>
+          <t>LYRIA</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>international</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -4848,25 +4848,25 @@
         </is>
       </c>
       <c r="G87" t="n">
+        <v>1040</v>
+      </c>
+      <c r="H87" t="n">
+        <v>0</v>
+      </c>
+      <c r="I87" t="n">
         <v>5</v>
       </c>
-      <c r="H87" t="n">
-        <v>0</v>
-      </c>
-      <c r="I87" t="n">
-        <v>0</v>
-      </c>
       <c r="J87" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="K87" t="n">
-        <v>0</v>
+        <v>112</v>
       </c>
       <c r="L87" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
       <c r="M87" t="n">
-        <v>0</v>
+        <v>1038</v>
       </c>
     </row>
     <row r="88">
@@ -4875,12 +4875,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Trenitalia</t>
+          <t>SNCF</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>EXP</t>
+          <t>TGV</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -4890,7 +4890,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -4899,25 +4899,25 @@
         </is>
       </c>
       <c r="G88" t="n">
-        <v>26</v>
+        <v>53</v>
       </c>
       <c r="H88" t="n">
         <v>0</v>
       </c>
       <c r="I88" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J88" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K88" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="L88" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="M88" t="n">
-        <v>24</v>
+        <v>53</v>
       </c>
     </row>
     <row r="89">
@@ -4926,22 +4926,22 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Trenitalia</t>
+          <t>SNCF</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>FA</t>
+          <t>TGV</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>domestic</t>
+          <t>international</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -4950,25 +4950,25 @@
         </is>
       </c>
       <c r="G89" t="n">
-        <v>476</v>
+        <v>1343</v>
       </c>
       <c r="H89" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="I89" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="J89" t="n">
-        <v>0</v>
+        <v>18</v>
       </c>
       <c r="K89" t="n">
-        <v>222</v>
+        <v>210</v>
       </c>
       <c r="L89" t="n">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="M89" t="n">
-        <v>476</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="90">
@@ -4977,12 +4977,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Trenitalia</t>
+          <t>SNCF</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>FB</t>
+          <t>TGV INOUI</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -4992,7 +4992,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -5001,25 +5001,25 @@
         </is>
       </c>
       <c r="G90" t="n">
-        <v>283</v>
+        <v>14774</v>
       </c>
       <c r="H90" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="I90" t="n">
-        <v>2</v>
+        <v>129</v>
       </c>
       <c r="J90" t="n">
-        <v>2</v>
+        <v>146</v>
       </c>
       <c r="K90" t="n">
-        <v>153</v>
+        <v>2042</v>
       </c>
       <c r="L90" t="n">
-        <v>75</v>
+        <v>943</v>
       </c>
       <c r="M90" t="n">
-        <v>283</v>
+        <v>14714</v>
       </c>
     </row>
     <row r="91">
@@ -5028,17 +5028,17 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Trenitalia</t>
+          <t>SNCF</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>TGV INOUI</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>domestic</t>
+          <t>international</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -5052,25 +5052,25 @@
         </is>
       </c>
       <c r="G91" t="n">
-        <v>6595</v>
+        <v>1140</v>
       </c>
       <c r="H91" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="I91" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="J91" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="K91" t="n">
-        <v>2071</v>
+        <v>271</v>
       </c>
       <c r="L91" t="n">
-        <v>942</v>
+        <v>143</v>
       </c>
       <c r="M91" t="n">
-        <v>6592</v>
+        <v>1122</v>
       </c>
     </row>
     <row r="92">
@@ -5084,44 +5084,44 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>FR</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>international</t>
+          <t>domestic</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G92" t="n">
-        <v>82</v>
+        <v>846</v>
       </c>
       <c r="H92" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I92" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J92" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="K92" t="n">
-        <v>49</v>
+        <v>180</v>
       </c>
       <c r="L92" t="n">
-        <v>19</v>
+        <v>64</v>
       </c>
       <c r="M92" t="n">
-        <v>77</v>
+        <v>837</v>
       </c>
     </row>
     <row r="93">
@@ -5135,12 +5135,12 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>IC</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>domestic</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
@@ -5150,29 +5150,29 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G93" t="n">
-        <v>2819</v>
+        <v>421</v>
       </c>
       <c r="H93" t="n">
         <v>0</v>
       </c>
       <c r="I93" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="J93" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="K93" t="n">
-        <v>786</v>
+        <v>0</v>
       </c>
       <c r="L93" t="n">
-        <v>334</v>
+        <v>0</v>
       </c>
       <c r="M93" t="n">
-        <v>2811</v>
+        <v>0</v>
       </c>
     </row>
     <row r="94">
@@ -5186,7 +5186,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>ICN</t>
+          <t>EN</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -5201,11 +5201,11 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G94" t="n">
-        <v>529</v>
+        <v>3</v>
       </c>
       <c r="H94" t="n">
         <v>0</v>
@@ -5217,13 +5217,13 @@
         <v>0</v>
       </c>
       <c r="K94" t="n">
-        <v>121</v>
+        <v>1</v>
       </c>
       <c r="L94" t="n">
-        <v>70</v>
+        <v>1</v>
       </c>
       <c r="M94" t="n">
-        <v>529</v>
+        <v>3</v>
       </c>
     </row>
     <row r="95">
@@ -5237,12 +5237,12 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>IR</t>
+          <t>EN</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>domestic</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -5252,29 +5252,29 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G95" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H95" t="n">
         <v>0</v>
       </c>
       <c r="I95" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J95" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K95" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="L95" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M95" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="96">
@@ -5288,7 +5288,7 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>MET</t>
+          <t>EXP</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -5303,29 +5303,29 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G96" t="n">
-        <v>6256</v>
+        <v>26</v>
       </c>
       <c r="H96" t="n">
         <v>0</v>
       </c>
       <c r="I96" t="n">
-        <v>110</v>
+        <v>2</v>
       </c>
       <c r="J96" t="n">
-        <v>110</v>
+        <v>2</v>
       </c>
       <c r="K96" t="n">
-        <v>171</v>
+        <v>13</v>
       </c>
       <c r="L96" t="n">
-        <v>42</v>
+        <v>9</v>
       </c>
       <c r="M96" t="n">
-        <v>6212</v>
+        <v>24</v>
       </c>
     </row>
     <row r="97">
@@ -5339,7 +5339,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>NCL</t>
+          <t>FA</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -5354,29 +5354,29 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G97" t="n">
-        <v>12</v>
+        <v>476</v>
       </c>
       <c r="H97" t="n">
         <v>0</v>
       </c>
       <c r="I97" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="J97" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K97" t="n">
-        <v>5</v>
+        <v>222</v>
       </c>
       <c r="L97" t="n">
-        <v>3</v>
+        <v>97</v>
       </c>
       <c r="M97" t="n">
-        <v>8</v>
+        <v>476</v>
       </c>
     </row>
     <row r="98">
@@ -5390,12 +5390,12 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>NCL</t>
+          <t>FB</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>domestic</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
@@ -5405,29 +5405,29 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G98" t="n">
+        <v>283</v>
+      </c>
+      <c r="H98" t="n">
+        <v>0</v>
+      </c>
+      <c r="I98" t="n">
         <v>2</v>
       </c>
-      <c r="H98" t="n">
-        <v>0</v>
-      </c>
-      <c r="I98" t="n">
-        <v>0</v>
-      </c>
       <c r="J98" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K98" t="n">
-        <v>0</v>
+        <v>153</v>
       </c>
       <c r="L98" t="n">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="M98" t="n">
-        <v>0</v>
+        <v>283</v>
       </c>
     </row>
     <row r="99">
@@ -5441,7 +5441,7 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>REG</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -5451,34 +5451,34 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G99" t="n">
-        <v>217367</v>
+        <v>6595</v>
       </c>
       <c r="H99" t="n">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="I99" t="n">
-        <v>4121</v>
+        <v>12</v>
       </c>
       <c r="J99" t="n">
-        <v>4156</v>
+        <v>12</v>
       </c>
       <c r="K99" t="n">
-        <v>22579</v>
+        <v>2071</v>
       </c>
       <c r="L99" t="n">
-        <v>5251</v>
+        <v>942</v>
       </c>
       <c r="M99" t="n">
-        <v>215098</v>
+        <v>6592</v>
       </c>
     </row>
     <row r="100">
@@ -5492,7 +5492,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>REG</t>
+          <t>FR</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -5502,34 +5502,34 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G100" t="n">
-        <v>1797</v>
+        <v>82</v>
       </c>
       <c r="H100" t="n">
         <v>0</v>
       </c>
       <c r="I100" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J100" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K100" t="n">
-        <v>95</v>
+        <v>49</v>
       </c>
       <c r="L100" t="n">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="M100" t="n">
-        <v>1794</v>
+        <v>77</v>
       </c>
     </row>
     <row r="101">
@@ -5543,12 +5543,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>REG</t>
+          <t>IC</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>domestic</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -5558,29 +5558,29 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G101" t="n">
-        <v>1</v>
+        <v>2819</v>
       </c>
       <c r="H101" t="n">
         <v>0</v>
       </c>
       <c r="I101" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="J101" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="K101" t="n">
-        <v>0</v>
+        <v>786</v>
       </c>
       <c r="L101" t="n">
-        <v>0</v>
+        <v>334</v>
       </c>
       <c r="M101" t="n">
-        <v>0</v>
+        <v>2811</v>
       </c>
     </row>
     <row r="102">
@@ -5589,12 +5589,12 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>UNKNOWN_OPERATOR</t>
+          <t>Trenitalia</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>BUS</t>
+          <t>ICN</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -5609,11 +5609,11 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G102" t="n">
-        <v>2943</v>
+        <v>529</v>
       </c>
       <c r="H102" t="n">
         <v>0</v>
@@ -5625,13 +5625,13 @@
         <v>0</v>
       </c>
       <c r="K102" t="n">
-        <v>0</v>
+        <v>121</v>
       </c>
       <c r="L102" t="n">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="M102" t="n">
-        <v>51</v>
+        <v>529</v>
       </c>
     </row>
     <row r="103">
@@ -5640,17 +5640,17 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>UNKNOWN_OPERATOR</t>
+          <t>Trenitalia</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>BUS</t>
+          <t>IR</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>international</t>
+          <t>domestic</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
@@ -5660,29 +5660,29 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G103" t="n">
-        <v>395</v>
+        <v>3</v>
       </c>
       <c r="H103" t="n">
         <v>0</v>
       </c>
       <c r="I103" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J103" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K103" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="L103" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M103" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="104">
@@ -5691,12 +5691,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>UNKNOWN_OPERATOR</t>
+          <t>Trenitalia</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Bus</t>
+          <t>MET</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -5715,25 +5715,25 @@
         </is>
       </c>
       <c r="G104" t="n">
-        <v>321</v>
+        <v>6256</v>
       </c>
       <c r="H104" t="n">
         <v>0</v>
       </c>
       <c r="I104" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="J104" t="n">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="K104" t="n">
-        <v>0</v>
+        <v>171</v>
       </c>
       <c r="L104" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="M104" t="n">
-        <v>0</v>
+        <v>6212</v>
       </c>
     </row>
     <row r="105">
@@ -5742,17 +5742,17 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>UNKNOWN_OPERATOR</t>
+          <t>Trenitalia</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Bus</t>
+          <t>NCL</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>international</t>
+          <t>domestic</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
@@ -5766,25 +5766,25 @@
         </is>
       </c>
       <c r="G105" t="n">
-        <v>759</v>
+        <v>12</v>
       </c>
       <c r="H105" t="n">
         <v>0</v>
       </c>
       <c r="I105" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J105" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K105" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L105" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M105" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="106">
@@ -5793,17 +5793,17 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>UNKNOWN_OPERATOR</t>
+          <t>Trenitalia</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>CAT</t>
+          <t>NCL</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>domestic</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -5817,7 +5817,7 @@
         </is>
       </c>
       <c r="G106" t="n">
-        <v>2021</v>
+        <v>2</v>
       </c>
       <c r="H106" t="n">
         <v>0</v>
@@ -5844,12 +5844,12 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>UNKNOWN_OPERATOR</t>
+          <t>Trenitalia</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>REG</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -5868,25 +5868,25 @@
         </is>
       </c>
       <c r="G107" t="n">
-        <v>1</v>
+        <v>217367</v>
       </c>
       <c r="H107" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="I107" t="n">
-        <v>0</v>
+        <v>4121</v>
       </c>
       <c r="J107" t="n">
-        <v>0</v>
+        <v>4156</v>
       </c>
       <c r="K107" t="n">
-        <v>0</v>
+        <v>22579</v>
       </c>
       <c r="L107" t="n">
-        <v>0</v>
+        <v>5251</v>
       </c>
       <c r="M107" t="n">
-        <v>0</v>
+        <v>215098</v>
       </c>
     </row>
     <row r="108">
@@ -5895,12 +5895,12 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>UNKNOWN_OPERATOR</t>
+          <t>Trenitalia</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>REG</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
@@ -5919,25 +5919,25 @@
         </is>
       </c>
       <c r="G108" t="n">
-        <v>582</v>
+        <v>1797</v>
       </c>
       <c r="H108" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I108" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J108" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="K108" t="n">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="L108" t="n">
-        <v>0</v>
+        <v>26</v>
       </c>
       <c r="M108" t="n">
-        <v>0</v>
+        <v>1794</v>
       </c>
     </row>
     <row r="109">
@@ -5946,17 +5946,17 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>UNKNOWN_OPERATOR</t>
+          <t>Trenitalia</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>DBK</t>
+          <t>REG</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>domestic</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -5970,7 +5970,7 @@
         </is>
       </c>
       <c r="G109" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H109" t="n">
         <v>0</v>
@@ -6002,7 +6002,7 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>EC</t>
+          <t>BUS</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -6021,7 +6021,7 @@
         </is>
       </c>
       <c r="G110" t="n">
-        <v>1</v>
+        <v>2943</v>
       </c>
       <c r="H110" t="n">
         <v>0</v>
@@ -6033,13 +6033,13 @@
         <v>0</v>
       </c>
       <c r="K110" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="L110" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M110" t="n">
-        <v>1</v>
+        <v>2943</v>
       </c>
     </row>
     <row r="111">
@@ -6053,7 +6053,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>EC</t>
+          <t>BUS</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
@@ -6072,25 +6072,25 @@
         </is>
       </c>
       <c r="G111" t="n">
-        <v>963</v>
+        <v>395</v>
       </c>
       <c r="H111" t="n">
         <v>0</v>
       </c>
       <c r="I111" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="J111" t="n">
-        <v>36</v>
+        <v>0</v>
       </c>
       <c r="K111" t="n">
-        <v>129</v>
+        <v>0</v>
       </c>
       <c r="L111" t="n">
-        <v>47</v>
+        <v>0</v>
       </c>
       <c r="M111" t="n">
-        <v>716</v>
+        <v>395</v>
       </c>
     </row>
     <row r="112">
@@ -6104,7 +6104,7 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>ECC</t>
+          <t>Bus</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -6123,25 +6123,25 @@
         </is>
       </c>
       <c r="G112" t="n">
-        <v>401</v>
+        <v>321</v>
       </c>
       <c r="H112" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="I112" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="J112" t="n">
-        <v>53</v>
+        <v>0</v>
       </c>
       <c r="K112" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="L112" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M112" t="n">
-        <v>192</v>
+        <v>321</v>
       </c>
     </row>
     <row r="113">
@@ -6155,7 +6155,7 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>ECC</t>
+          <t>Bus</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="G113" t="n">
-        <v>64</v>
+        <v>759</v>
       </c>
       <c r="H113" t="n">
         <v>0</v>
@@ -6192,7 +6192,7 @@
         <v>0</v>
       </c>
       <c r="M113" t="n">
-        <v>0</v>
+        <v>759</v>
       </c>
     </row>
     <row r="114">
@@ -6206,12 +6206,12 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>ECC</t>
+          <t>CAT</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>domestic</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
@@ -6225,16 +6225,16 @@
         </is>
       </c>
       <c r="G114" t="n">
-        <v>317</v>
+        <v>2021</v>
       </c>
       <c r="H114" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="I114" t="n">
         <v>0</v>
       </c>
       <c r="J114" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="K114" t="n">
         <v>0</v>
@@ -6243,7 +6243,7 @@
         <v>0</v>
       </c>
       <c r="M114" t="n">
-        <v>0</v>
+        <v>2021</v>
       </c>
     </row>
     <row r="115">
@@ -6257,7 +6257,7 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>ECD</t>
+          <t>D</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -6276,25 +6276,25 @@
         </is>
       </c>
       <c r="G115" t="n">
-        <v>85</v>
+        <v>1</v>
       </c>
       <c r="H115" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="I115" t="n">
         <v>0</v>
       </c>
       <c r="J115" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="K115" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L115" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M115" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
     </row>
     <row r="116">
@@ -6308,7 +6308,7 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>ECD</t>
+          <t>D</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -6327,25 +6327,25 @@
         </is>
       </c>
       <c r="G116" t="n">
-        <v>731</v>
+        <v>582</v>
       </c>
       <c r="H116" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="I116" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J116" t="n">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="K116" t="n">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="L116" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="M116" t="n">
-        <v>541</v>
+        <v>572</v>
       </c>
     </row>
     <row r="117">
@@ -6359,12 +6359,12 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>ECD</t>
+          <t>DBK</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>domestic</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -6378,7 +6378,7 @@
         </is>
       </c>
       <c r="G117" t="n">
-        <v>64</v>
+        <v>2</v>
       </c>
       <c r="H117" t="n">
         <v>0</v>
@@ -6390,13 +6390,13 @@
         <v>0</v>
       </c>
       <c r="K117" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L117" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M117" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="118">
@@ -6410,7 +6410,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>EN</t>
+          <t>EC</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -6429,25 +6429,25 @@
         </is>
       </c>
       <c r="G118" t="n">
-        <v>14</v>
+        <v>267</v>
       </c>
       <c r="H118" t="n">
         <v>0</v>
       </c>
       <c r="I118" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J118" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K118" t="n">
-        <v>0</v>
+        <v>31</v>
       </c>
       <c r="L118" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="M118" t="n">
-        <v>0</v>
+        <v>262</v>
       </c>
     </row>
     <row r="119">
@@ -6461,12 +6461,12 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>GEP</t>
+          <t>EN</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>domestic</t>
+          <t>international</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -6480,7 +6480,7 @@
         </is>
       </c>
       <c r="G119" t="n">
-        <v>56</v>
+        <v>14</v>
       </c>
       <c r="H119" t="n">
         <v>0</v>
@@ -6492,13 +6492,13 @@
         <v>0</v>
       </c>
       <c r="K119" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L119" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="M119" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
     </row>
     <row r="120">
@@ -6517,7 +6517,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>international</t>
+          <t>domestic</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
@@ -6549,7 +6549,7 @@
         <v>0</v>
       </c>
       <c r="M120" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
     </row>
     <row r="121">
@@ -6563,7 +6563,7 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>IC</t>
+          <t>GEP</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -6582,7 +6582,7 @@
         </is>
       </c>
       <c r="G121" t="n">
-        <v>141</v>
+        <v>56</v>
       </c>
       <c r="H121" t="n">
         <v>0</v>
@@ -6600,7 +6600,7 @@
         <v>0</v>
       </c>
       <c r="M121" t="n">
-        <v>0</v>
+        <v>56</v>
       </c>
     </row>
     <row r="122">
@@ -6614,12 +6614,12 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>INT</t>
+          <t>IC</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>international</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
@@ -6633,25 +6633,25 @@
         </is>
       </c>
       <c r="G122" t="n">
+        <v>141</v>
+      </c>
+      <c r="H122" t="n">
+        <v>0</v>
+      </c>
+      <c r="I122" t="n">
         <v>1</v>
       </c>
-      <c r="H122" t="n">
-        <v>0</v>
-      </c>
-      <c r="I122" t="n">
-        <v>0</v>
-      </c>
       <c r="J122" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K122" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="L122" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M122" t="n">
-        <v>0</v>
+        <v>139</v>
       </c>
     </row>
     <row r="123">
@@ -6665,12 +6665,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>IR</t>
+          <t>INT</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>domestic</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
@@ -6684,16 +6684,16 @@
         </is>
       </c>
       <c r="G123" t="n">
-        <v>9983</v>
+        <v>1</v>
       </c>
       <c r="H123" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I123" t="n">
-        <v>58</v>
+        <v>0</v>
       </c>
       <c r="J123" t="n">
-        <v>63</v>
+        <v>0</v>
       </c>
       <c r="K123" t="n">
         <v>0</v>
@@ -6721,7 +6721,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>international</t>
+          <t>domestic</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -6735,25 +6735,25 @@
         </is>
       </c>
       <c r="G124" t="n">
-        <v>20</v>
+        <v>9983</v>
       </c>
       <c r="H124" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I124" t="n">
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="J124" t="n">
-        <v>0</v>
+        <v>68</v>
       </c>
       <c r="K124" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L124" t="n">
         <v>0</v>
       </c>
       <c r="M124" t="n">
-        <v>0</v>
+        <v>9920</v>
       </c>
     </row>
     <row r="125">
@@ -6767,12 +6767,12 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>PE</t>
+          <t>IR</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>domestic</t>
+          <t>international</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
@@ -6786,7 +6786,7 @@
         </is>
       </c>
       <c r="G125" t="n">
-        <v>1318</v>
+        <v>20</v>
       </c>
       <c r="H125" t="n">
         <v>0</v>
@@ -6804,7 +6804,7 @@
         <v>0</v>
       </c>
       <c r="M125" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
     </row>
     <row r="126">
@@ -6823,7 +6823,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>international</t>
+          <t>domestic</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
@@ -6837,7 +6837,7 @@
         </is>
       </c>
       <c r="G126" t="n">
-        <v>50</v>
+        <v>1318</v>
       </c>
       <c r="H126" t="n">
         <v>0</v>
@@ -6855,7 +6855,7 @@
         <v>0</v>
       </c>
       <c r="M126" t="n">
-        <v>0</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="127">
@@ -6864,17 +6864,17 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Westbahn</t>
+          <t>UNKNOWN_OPERATOR</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>WB</t>
+          <t>PE</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>domestic</t>
+          <t>international</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
@@ -6884,11 +6884,11 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G127" t="n">
-        <v>1366</v>
+        <v>50</v>
       </c>
       <c r="H127" t="n">
         <v>0</v>
@@ -6906,7 +6906,7 @@
         <v>0</v>
       </c>
       <c r="M127" t="n">
-        <v>0</v>
+        <v>50</v>
       </c>
     </row>
     <row r="128">
@@ -6925,39 +6925,90 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
+          <t>domestic</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G128" t="n">
+        <v>1366</v>
+      </c>
+      <c r="H128" t="n">
+        <v>0</v>
+      </c>
+      <c r="I128" t="n">
+        <v>0</v>
+      </c>
+      <c r="J128" t="n">
+        <v>0</v>
+      </c>
+      <c r="K128" t="n">
+        <v>26</v>
+      </c>
+      <c r="L128" t="n">
+        <v>13</v>
+      </c>
+      <c r="M128" t="n">
+        <v>1366</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Westbahn</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>WB</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
           <t>international</t>
         </is>
       </c>
-      <c r="E128" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="F128" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="G128" t="n">
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G129" t="n">
         <v>4</v>
       </c>
-      <c r="H128" t="n">
-        <v>0</v>
-      </c>
-      <c r="I128" t="n">
-        <v>0</v>
-      </c>
-      <c r="J128" t="n">
-        <v>0</v>
-      </c>
-      <c r="K128" t="n">
-        <v>0</v>
-      </c>
-      <c r="L128" t="n">
-        <v>0</v>
-      </c>
-      <c r="M128" t="n">
-        <v>0</v>
+      <c r="H129" t="n">
+        <v>0</v>
+      </c>
+      <c r="I129" t="n">
+        <v>0</v>
+      </c>
+      <c r="J129" t="n">
+        <v>0</v>
+      </c>
+      <c r="K129" t="n">
+        <v>1</v>
+      </c>
+      <c r="L129" t="n">
+        <v>0</v>
+      </c>
+      <c r="M129" t="n">
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>